<commit_message>
add debug_mode for VT7
</commit_message>
<xml_diff>
--- a/__docs/trade_data.xlsx
+++ b/__docs/trade_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter3\__docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9E9DD6C-CC1A-4119-9DCE-2A013E25D48B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2525A5C4-1803-469C-8A55-F74E7C44C991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2880,13 +2880,13 @@
         <v>132</v>
       </c>
       <c r="C2">
-        <v>-1.9</v>
+        <v>-23.9</v>
       </c>
       <c r="D2">
-        <v>-0.38</v>
+        <v>-4.7799999999999994</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -2895,7 +2895,7 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I2" s="11">
         <f>IFERROR((F2/E2)*100,0)</f>
@@ -2903,23 +2903,23 @@
       </c>
       <c r="J2" s="14">
         <f>IFERROR(C2/E2,0)</f>
-        <v>-1.9</v>
+        <v>-11.95</v>
       </c>
       <c r="K2" s="14">
         <f>IFERROR(D2/E2,0)</f>
-        <v>-0.38</v>
+        <v>-2.3899999999999997</v>
       </c>
       <c r="M2">
         <f t="shared" ref="M2:R2" si="0">C2+T2</f>
-        <v>-1.9</v>
+        <v>-23.9</v>
       </c>
       <c r="N2">
         <f t="shared" si="0"/>
-        <v>-0.38</v>
+        <v>-4.7799999999999994</v>
       </c>
       <c r="O2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P2">
         <f t="shared" si="0"/>
@@ -2931,7 +2931,7 @@
       </c>
       <c r="R2">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
@@ -3004,13 +3004,13 @@
         <v>135</v>
       </c>
       <c r="C4">
-        <v>-2.7</v>
+        <v>-20.9</v>
       </c>
       <c r="D4">
-        <v>-0.54</v>
+        <v>-4.18</v>
       </c>
       <c r="E4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -3019,31 +3019,31 @@
         <v>0</v>
       </c>
       <c r="H4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I4" s="11">
         <f t="shared" si="1"/>
-        <v>33.333333333333329</v>
+        <v>20</v>
       </c>
       <c r="J4" s="14">
         <f t="shared" si="2"/>
-        <v>-0.9</v>
+        <v>-4.18</v>
       </c>
       <c r="K4" s="14">
         <f t="shared" si="3"/>
-        <v>-0.18000000000000002</v>
+        <v>-0.83599999999999997</v>
       </c>
       <c r="M4">
         <f t="shared" si="4"/>
-        <v>-2.7</v>
+        <v>-20.9</v>
       </c>
       <c r="N4">
         <f t="shared" si="5"/>
-        <v>-0.54</v>
+        <v>-4.18</v>
       </c>
       <c r="O4">
         <f t="shared" si="6"/>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P4">
         <f t="shared" si="7"/>
@@ -3055,7 +3055,7 @@
       </c>
       <c r="R4">
         <f t="shared" si="9"/>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
@@ -3128,16 +3128,16 @@
         <v>134</v>
       </c>
       <c r="C6">
-        <v>-2.5</v>
+        <v>-1.9</v>
       </c>
       <c r="D6">
-        <v>-0.5</v>
+        <v>-0.38</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -3147,31 +3147,31 @@
       </c>
       <c r="I6" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J6" s="14">
         <f t="shared" si="2"/>
-        <v>-2.5</v>
+        <v>-0.95</v>
       </c>
       <c r="K6" s="14">
         <f t="shared" si="3"/>
-        <v>-0.5</v>
+        <v>-0.19</v>
       </c>
       <c r="M6">
         <f t="shared" si="4"/>
-        <v>-2.5</v>
+        <v>-1.9</v>
       </c>
       <c r="N6">
         <f t="shared" si="5"/>
-        <v>-0.5</v>
+        <v>-0.38</v>
       </c>
       <c r="O6">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P6">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q6">
         <f t="shared" si="8"/>
@@ -3438,50 +3438,50 @@
         <v>72</v>
       </c>
       <c r="C11">
-        <v>30.1</v>
+        <v>19.2</v>
       </c>
       <c r="D11">
-        <v>6.0200000000000005</v>
+        <v>3.8400000000000003</v>
       </c>
       <c r="E11">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F11">
+        <v>6</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
         <v>5</v>
       </c>
-      <c r="G11">
-        <v>0</v>
-      </c>
-      <c r="H11">
-        <v>3</v>
-      </c>
       <c r="I11" s="11">
         <f t="shared" si="1"/>
-        <v>62.5</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="J11" s="14">
         <f t="shared" si="2"/>
-        <v>3.7625000000000002</v>
+        <v>1.7454545454545454</v>
       </c>
       <c r="K11" s="14">
         <f t="shared" si="3"/>
-        <v>0.75250000000000006</v>
+        <v>0.34909090909090912</v>
       </c>
       <c r="M11">
         <f t="shared" si="4"/>
-        <v>30.1</v>
+        <v>19.2</v>
       </c>
       <c r="N11">
         <f t="shared" si="5"/>
-        <v>6.0200000000000005</v>
+        <v>3.8400000000000003</v>
       </c>
       <c r="O11">
         <f t="shared" si="6"/>
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="P11">
         <f t="shared" si="7"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q11">
         <f t="shared" si="8"/>
@@ -3489,7 +3489,7 @@
       </c>
       <c r="R11">
         <f t="shared" si="9"/>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
@@ -3624,50 +3624,50 @@
         <v>60</v>
       </c>
       <c r="C14">
-        <v>36.799999999999997</v>
+        <v>24.4</v>
       </c>
       <c r="D14">
-        <v>7.36</v>
+        <v>4.8800000000000008</v>
       </c>
       <c r="E14">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F14">
+        <v>6</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
         <v>5</v>
       </c>
-      <c r="G14">
-        <v>0</v>
-      </c>
-      <c r="H14">
-        <v>4</v>
-      </c>
       <c r="I14" s="11">
         <f t="shared" si="1"/>
-        <v>55.555555555555557</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="J14" s="14">
         <f t="shared" si="2"/>
-        <v>4.0888888888888886</v>
+        <v>2.2181818181818183</v>
       </c>
       <c r="K14" s="14">
         <f t="shared" si="3"/>
-        <v>0.81777777777777783</v>
+        <v>0.44363636363636372</v>
       </c>
       <c r="M14">
         <f t="shared" si="4"/>
-        <v>36.799999999999997</v>
+        <v>24.4</v>
       </c>
       <c r="N14">
         <f t="shared" si="5"/>
-        <v>7.36</v>
+        <v>4.8800000000000008</v>
       </c>
       <c r="O14">
         <f t="shared" si="6"/>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P14">
         <f t="shared" si="7"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q14">
         <f t="shared" si="8"/>
@@ -3675,7 +3675,7 @@
       </c>
       <c r="R14">
         <f t="shared" si="9"/>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
@@ -3686,16 +3686,16 @@
         <v>67</v>
       </c>
       <c r="C15">
-        <v>11</v>
+        <v>15.4</v>
       </c>
       <c r="D15">
-        <v>2.2000000000000002</v>
+        <v>3.08</v>
       </c>
       <c r="E15">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F15">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G15">
         <v>0</v>
@@ -3705,31 +3705,31 @@
       </c>
       <c r="I15" s="11">
         <f t="shared" si="1"/>
-        <v>66.666666666666657</v>
+        <v>70</v>
       </c>
       <c r="J15" s="14">
         <f t="shared" si="2"/>
-        <v>1.2222222222222223</v>
+        <v>1.54</v>
       </c>
       <c r="K15" s="14">
         <f t="shared" si="3"/>
-        <v>0.24444444444444446</v>
+        <v>0.308</v>
       </c>
       <c r="M15">
         <f t="shared" si="4"/>
-        <v>11</v>
+        <v>15.4</v>
       </c>
       <c r="N15">
         <f t="shared" si="5"/>
-        <v>2.2000000000000002</v>
+        <v>3.08</v>
       </c>
       <c r="O15">
         <f t="shared" si="6"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P15">
         <f t="shared" si="7"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q15">
         <f t="shared" si="8"/>
@@ -3996,16 +3996,16 @@
         <v>69</v>
       </c>
       <c r="C20">
-        <v>5.6999999999999984</v>
+        <v>7.6999999999999984</v>
       </c>
       <c r="D20">
-        <v>1.1399999999999997</v>
+        <v>1.5399999999999996</v>
       </c>
       <c r="E20">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F20">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G20">
         <v>1</v>
@@ -4015,31 +4015,31 @@
       </c>
       <c r="I20" s="11">
         <f t="shared" si="1"/>
-        <v>43.478260869565219</v>
+        <v>48</v>
       </c>
       <c r="J20" s="14">
         <f t="shared" si="2"/>
-        <v>0.24782608695652167</v>
+        <v>0.30799999999999994</v>
       </c>
       <c r="K20" s="14">
         <f t="shared" si="3"/>
-        <v>4.9565217391304331E-2</v>
+        <v>6.1599999999999981E-2</v>
       </c>
       <c r="M20">
         <f t="shared" si="4"/>
-        <v>5.6999999999999984</v>
+        <v>7.6999999999999984</v>
       </c>
       <c r="N20">
         <f t="shared" si="10"/>
-        <v>1.1399999999999997</v>
+        <v>1.5399999999999996</v>
       </c>
       <c r="O20">
         <f t="shared" si="11"/>
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="P20">
         <f t="shared" si="12"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="Q20">
         <f t="shared" si="13"/>
@@ -4120,13 +4120,13 @@
         <v>121</v>
       </c>
       <c r="C22">
-        <v>1.2</v>
+        <v>-1.9000000000000001</v>
       </c>
       <c r="D22">
-        <v>0.24</v>
+        <v>-0.38</v>
       </c>
       <c r="E22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22">
         <v>1</v>
@@ -4135,31 +4135,31 @@
         <v>0</v>
       </c>
       <c r="H22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I22" s="11">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="J22" s="14">
         <f t="shared" si="2"/>
-        <v>1.2</v>
+        <v>-0.95000000000000007</v>
       </c>
       <c r="K22" s="14">
         <f t="shared" si="3"/>
-        <v>0.24</v>
+        <v>-0.19</v>
       </c>
       <c r="M22">
         <f t="shared" si="4"/>
-        <v>1.2</v>
+        <v>-1.9000000000000001</v>
       </c>
       <c r="N22">
         <f t="shared" si="10"/>
-        <v>0.24</v>
+        <v>-0.38</v>
       </c>
       <c r="O22">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P22">
         <f t="shared" si="12"/>
@@ -4171,7 +4171,7 @@
       </c>
       <c r="R22">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.25">
@@ -4182,13 +4182,13 @@
         <v>66</v>
       </c>
       <c r="C23">
-        <v>5.7</v>
+        <v>3.3000000000000003</v>
       </c>
       <c r="D23">
-        <v>1.1400000000000001</v>
+        <v>0.66000000000000014</v>
       </c>
       <c r="E23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F23">
         <v>3</v>
@@ -4197,31 +4197,31 @@
         <v>0</v>
       </c>
       <c r="H23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I23" s="11">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="J23" s="14">
         <f t="shared" si="2"/>
-        <v>1.1400000000000001</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="K23" s="14">
         <f t="shared" si="3"/>
-        <v>0.22800000000000004</v>
+        <v>0.11000000000000003</v>
       </c>
       <c r="M23">
         <f t="shared" si="4"/>
-        <v>5.7</v>
+        <v>3.3000000000000003</v>
       </c>
       <c r="N23">
         <f t="shared" si="10"/>
-        <v>1.1400000000000001</v>
+        <v>0.66000000000000014</v>
       </c>
       <c r="O23">
         <f t="shared" si="11"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P23">
         <f t="shared" si="12"/>
@@ -4233,7 +4233,7 @@
       </c>
       <c r="R23">
         <f t="shared" si="14"/>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
@@ -4430,50 +4430,50 @@
         <v>70</v>
       </c>
       <c r="C27">
-        <v>36.9</v>
+        <v>31.4</v>
       </c>
       <c r="D27">
-        <v>7.3800000000000008</v>
+        <v>6.2800000000000011</v>
       </c>
       <c r="E27">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F27">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G27">
         <v>0</v>
       </c>
       <c r="H27">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I27" s="11">
         <f t="shared" si="1"/>
-        <v>71.428571428571431</v>
+        <v>57.894736842105267</v>
       </c>
       <c r="J27" s="14">
         <f t="shared" si="2"/>
-        <v>2.6357142857142857</v>
+        <v>1.6526315789473685</v>
       </c>
       <c r="K27" s="14">
         <f t="shared" si="3"/>
-        <v>0.52714285714285725</v>
+        <v>0.33052631578947372</v>
       </c>
       <c r="M27">
         <f t="shared" si="4"/>
-        <v>36.9</v>
+        <v>31.4</v>
       </c>
       <c r="N27">
         <f t="shared" si="10"/>
-        <v>7.3800000000000008</v>
+        <v>6.2800000000000011</v>
       </c>
       <c r="O27">
         <f t="shared" si="11"/>
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="P27">
         <f t="shared" si="12"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q27">
         <f t="shared" si="13"/>
@@ -4481,7 +4481,7 @@
       </c>
       <c r="R27">
         <f t="shared" si="14"/>
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
@@ -4616,13 +4616,13 @@
         <v>128</v>
       </c>
       <c r="C30">
-        <v>0.3</v>
+        <v>-3.5</v>
       </c>
       <c r="D30">
-        <v>0.06</v>
+        <v>-0.7</v>
       </c>
       <c r="E30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30">
         <v>1</v>
@@ -4631,31 +4631,31 @@
         <v>0</v>
       </c>
       <c r="H30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I30" s="11">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="J30" s="14">
         <f t="shared" si="2"/>
-        <v>0.3</v>
+        <v>-1.75</v>
       </c>
       <c r="K30" s="14">
         <f t="shared" si="3"/>
-        <v>0.06</v>
+        <v>-0.35</v>
       </c>
       <c r="M30">
         <f t="shared" si="4"/>
-        <v>0.3</v>
+        <v>-3.5</v>
       </c>
       <c r="N30">
         <f t="shared" si="10"/>
-        <v>0.06</v>
+        <v>-0.7</v>
       </c>
       <c r="O30">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P30">
         <f t="shared" si="12"/>
@@ -4667,7 +4667,7 @@
       </c>
       <c r="R30">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.25">
@@ -4740,16 +4740,16 @@
         <v>124</v>
       </c>
       <c r="C32">
-        <v>0.9</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="D32">
-        <v>0.18</v>
+        <v>0.22</v>
       </c>
       <c r="E32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G32">
         <v>0</v>
@@ -4763,27 +4763,27 @@
       </c>
       <c r="J32" s="14">
         <f t="shared" si="2"/>
-        <v>0.9</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="K32" s="14">
         <f t="shared" si="3"/>
-        <v>0.18</v>
+        <v>0.11</v>
       </c>
       <c r="M32">
         <f t="shared" si="4"/>
-        <v>0.9</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="N32">
         <f t="shared" si="10"/>
-        <v>0.18</v>
+        <v>0.22</v>
       </c>
       <c r="O32">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P32">
         <f t="shared" si="12"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q32">
         <f t="shared" si="13"/>
@@ -4802,16 +4802,16 @@
         <v>127</v>
       </c>
       <c r="C33">
-        <v>-10</v>
+        <v>-1.1999999999999993</v>
       </c>
       <c r="D33">
-        <v>-2</v>
+        <v>-0.24</v>
       </c>
       <c r="E33">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33">
         <v>0</v>
@@ -4821,31 +4821,31 @@
       </c>
       <c r="I33" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J33" s="14">
         <f t="shared" si="2"/>
-        <v>-10</v>
+        <v>-0.59999999999999964</v>
       </c>
       <c r="K33" s="14">
         <f t="shared" si="3"/>
-        <v>-2</v>
+        <v>-0.12</v>
       </c>
       <c r="M33">
         <f t="shared" si="4"/>
-        <v>-10</v>
+        <v>-1.1999999999999993</v>
       </c>
       <c r="N33">
         <f t="shared" si="10"/>
-        <v>-2</v>
+        <v>-0.24</v>
       </c>
       <c r="O33">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P33">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q33">
         <f t="shared" si="13"/>
@@ -4926,13 +4926,13 @@
         <v>131</v>
       </c>
       <c r="C35">
-        <v>2.2999999999999998</v>
+        <v>-0.40000000000000036</v>
       </c>
       <c r="D35">
-        <v>0.45999999999999996</v>
+        <v>-8.0000000000000071E-2</v>
       </c>
       <c r="E35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F35">
         <v>1</v>
@@ -4941,31 +4941,31 @@
         <v>0</v>
       </c>
       <c r="H35">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I35" s="11">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="J35" s="14">
         <f t="shared" si="2"/>
-        <v>2.2999999999999998</v>
+        <v>-0.20000000000000018</v>
       </c>
       <c r="K35" s="14">
         <f t="shared" si="3"/>
-        <v>0.45999999999999996</v>
+        <v>-4.0000000000000036E-2</v>
       </c>
       <c r="M35">
         <f t="shared" si="4"/>
-        <v>2.2999999999999998</v>
+        <v>-0.40000000000000036</v>
       </c>
       <c r="N35">
         <f t="shared" si="10"/>
-        <v>0.45999999999999996</v>
+        <v>-8.0000000000000071E-2</v>
       </c>
       <c r="O35">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P35">
         <f t="shared" si="12"/>
@@ -4977,7 +4977,7 @@
       </c>
       <c r="R35">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.25">
@@ -5236,46 +5236,46 @@
         <v>87</v>
       </c>
       <c r="C40">
-        <v>-3.4</v>
+        <v>-6.5</v>
       </c>
       <c r="D40">
-        <v>-0.67999999999999994</v>
+        <v>-1.2999999999999998</v>
       </c>
       <c r="E40">
+        <v>4</v>
+      </c>
+      <c r="F40">
+        <v>1</v>
+      </c>
+      <c r="G40">
+        <v>0</v>
+      </c>
+      <c r="H40">
         <v>3</v>
       </c>
-      <c r="F40">
-        <v>1</v>
-      </c>
-      <c r="G40">
-        <v>0</v>
-      </c>
-      <c r="H40">
-        <v>2</v>
-      </c>
       <c r="I40" s="11">
         <f t="shared" si="1"/>
-        <v>33.333333333333329</v>
+        <v>25</v>
       </c>
       <c r="J40" s="14">
         <f t="shared" si="2"/>
-        <v>-1.1333333333333333</v>
+        <v>-1.625</v>
       </c>
       <c r="K40" s="14">
         <f t="shared" si="3"/>
-        <v>-0.22666666666666666</v>
+        <v>-0.32499999999999996</v>
       </c>
       <c r="M40">
         <f t="shared" si="4"/>
-        <v>-3.4</v>
+        <v>-6.5</v>
       </c>
       <c r="N40">
         <f t="shared" si="10"/>
-        <v>-0.67999999999999994</v>
+        <v>-1.2999999999999998</v>
       </c>
       <c r="O40">
         <f t="shared" si="11"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P40">
         <f t="shared" si="12"/>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="R40">
         <f t="shared" si="14"/>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.25">
@@ -5484,13 +5484,13 @@
         <v>79</v>
       </c>
       <c r="C44">
-        <v>12.4</v>
+        <v>1.9000000000000004</v>
       </c>
       <c r="D44">
-        <v>2.48</v>
+        <v>0.37999999999999989</v>
       </c>
       <c r="E44">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F44">
         <v>3</v>
@@ -5499,31 +5499,31 @@
         <v>0</v>
       </c>
       <c r="H44">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I44" s="11">
         <f t="shared" si="1"/>
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="J44" s="14">
         <f t="shared" si="2"/>
-        <v>3.1</v>
+        <v>0.38000000000000006</v>
       </c>
       <c r="K44" s="14">
         <f t="shared" si="3"/>
-        <v>0.62</v>
+        <v>7.5999999999999984E-2</v>
       </c>
       <c r="M44">
         <f t="shared" si="4"/>
-        <v>12.4</v>
+        <v>1.9000000000000004</v>
       </c>
       <c r="N44">
         <f t="shared" si="10"/>
-        <v>2.48</v>
+        <v>0.37999999999999989</v>
       </c>
       <c r="O44">
         <f t="shared" si="11"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P44">
         <f t="shared" si="12"/>
@@ -5535,7 +5535,7 @@
       </c>
       <c r="R44">
         <f t="shared" si="14"/>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.25">
@@ -5856,13 +5856,13 @@
         <v>108</v>
       </c>
       <c r="C50">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="D50">
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="E50">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F50">
         <v>0</v>
@@ -5871,7 +5871,7 @@
         <v>0</v>
       </c>
       <c r="H50">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I50" s="11">
         <f t="shared" si="1"/>
@@ -5879,23 +5879,23 @@
       </c>
       <c r="J50" s="14">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="K50" s="14">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="M50">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="N50">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="O50">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P50">
         <f t="shared" si="12"/>
@@ -5907,7 +5907,7 @@
       </c>
       <c r="R50">
         <f t="shared" ref="R50:R67" si="16">H50+Y50</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:18" x14ac:dyDescent="0.25">
@@ -6042,13 +6042,13 @@
         <v>78</v>
       </c>
       <c r="C53">
-        <v>1.7</v>
+        <v>-2.8999999999999995</v>
       </c>
       <c r="D53">
-        <v>0.33999999999999997</v>
+        <v>-0.57999999999999996</v>
       </c>
       <c r="E53">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F53">
         <v>1</v>
@@ -6057,31 +6057,31 @@
         <v>0</v>
       </c>
       <c r="H53">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I53" s="11">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="J53" s="14">
         <f t="shared" si="2"/>
-        <v>1.7</v>
+        <v>-1.4499999999999997</v>
       </c>
       <c r="K53" s="14">
         <f t="shared" si="3"/>
-        <v>0.33999999999999997</v>
+        <v>-0.28999999999999998</v>
       </c>
       <c r="M53">
         <f t="shared" si="4"/>
-        <v>1.7</v>
+        <v>-2.8999999999999995</v>
       </c>
       <c r="N53">
         <f t="shared" si="10"/>
-        <v>0.33999999999999997</v>
+        <v>-0.57999999999999996</v>
       </c>
       <c r="O53">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P53">
         <f t="shared" si="12"/>
@@ -6093,7 +6093,7 @@
       </c>
       <c r="R53">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:18" x14ac:dyDescent="0.25">
@@ -6166,16 +6166,16 @@
         <v>73</v>
       </c>
       <c r="C55">
-        <v>-5.7999999999999989</v>
+        <v>1.6000000000000014</v>
       </c>
       <c r="D55">
-        <v>-1.1599999999999999</v>
+        <v>0.32000000000000006</v>
       </c>
       <c r="E55">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F55">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G55">
         <v>0</v>
@@ -6185,31 +6185,31 @@
       </c>
       <c r="I55" s="11">
         <f t="shared" si="1"/>
-        <v>20</v>
+        <v>33.333333333333329</v>
       </c>
       <c r="J55" s="14">
         <f t="shared" si="2"/>
-        <v>-1.1599999999999997</v>
+        <v>0.26666666666666689</v>
       </c>
       <c r="K55" s="14">
         <f t="shared" si="3"/>
-        <v>-0.23199999999999998</v>
+        <v>5.3333333333333344E-2</v>
       </c>
       <c r="M55">
         <f t="shared" si="4"/>
-        <v>-5.7999999999999989</v>
+        <v>1.6000000000000014</v>
       </c>
       <c r="N55">
         <f t="shared" si="10"/>
-        <v>-1.1599999999999999</v>
+        <v>0.32000000000000006</v>
       </c>
       <c r="O55">
         <f t="shared" si="11"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P55">
         <f t="shared" si="12"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q55">
         <f t="shared" si="15"/>
@@ -6662,13 +6662,13 @@
         <v>62</v>
       </c>
       <c r="C63">
-        <v>2.8</v>
+        <v>-14.3</v>
       </c>
       <c r="D63">
-        <v>0.56000000000000005</v>
+        <v>-2.86</v>
       </c>
       <c r="E63">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F63">
         <v>7</v>
@@ -6677,31 +6677,31 @@
         <v>0</v>
       </c>
       <c r="H63">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I63" s="11">
         <f t="shared" si="1"/>
-        <v>50</v>
+        <v>46.666666666666664</v>
       </c>
       <c r="J63" s="14">
         <f t="shared" si="2"/>
-        <v>0.19999999999999998</v>
+        <v>-0.95333333333333337</v>
       </c>
       <c r="K63" s="14">
         <f t="shared" si="3"/>
-        <v>0.04</v>
+        <v>-0.19066666666666665</v>
       </c>
       <c r="M63">
         <f t="shared" si="4"/>
-        <v>2.8</v>
+        <v>-14.3</v>
       </c>
       <c r="N63">
         <f t="shared" si="10"/>
-        <v>0.56000000000000005</v>
+        <v>-2.86</v>
       </c>
       <c r="O63">
         <f t="shared" si="11"/>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P63">
         <f t="shared" si="12"/>
@@ -6713,7 +6713,7 @@
       </c>
       <c r="R63">
         <f t="shared" si="16"/>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="64" spans="1:18" x14ac:dyDescent="0.25">
@@ -6724,50 +6724,50 @@
         <v>61</v>
       </c>
       <c r="C64">
-        <v>35.5</v>
+        <v>32.6</v>
       </c>
       <c r="D64">
-        <v>7.1000000000000005</v>
+        <v>6.5200000000000005</v>
       </c>
       <c r="E64">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F64">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G64">
         <v>0</v>
       </c>
       <c r="H64">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I64" s="11">
         <f t="shared" si="1"/>
-        <v>76.19047619047619</v>
+        <v>70.833333333333343</v>
       </c>
       <c r="J64" s="14">
         <f t="shared" si="2"/>
-        <v>1.6904761904761905</v>
+        <v>1.3583333333333334</v>
       </c>
       <c r="K64" s="14">
         <f t="shared" si="3"/>
-        <v>0.33809523809523812</v>
+        <v>0.27166666666666667</v>
       </c>
       <c r="M64">
         <f t="shared" si="4"/>
-        <v>35.5</v>
+        <v>32.6</v>
       </c>
       <c r="N64">
         <f t="shared" si="10"/>
-        <v>7.1000000000000005</v>
+        <v>6.5200000000000005</v>
       </c>
       <c r="O64">
         <f t="shared" si="11"/>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="P64">
         <f t="shared" si="12"/>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q64">
         <f t="shared" si="15"/>
@@ -6775,7 +6775,7 @@
       </c>
       <c r="R64">
         <f t="shared" si="16"/>
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="65" spans="1:18" x14ac:dyDescent="0.25">
@@ -6848,13 +6848,13 @@
         <v>63</v>
       </c>
       <c r="C66">
-        <v>28.4</v>
+        <v>17.5</v>
       </c>
       <c r="D66">
-        <v>5.68</v>
+        <v>3.4999999999999996</v>
       </c>
       <c r="E66">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F66">
         <v>6</v>
@@ -6863,31 +6863,31 @@
         <v>1</v>
       </c>
       <c r="H66">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I66" s="11">
         <f t="shared" si="1"/>
-        <v>66.666666666666657</v>
+        <v>60</v>
       </c>
       <c r="J66" s="14">
         <f t="shared" si="2"/>
-        <v>3.1555555555555554</v>
+        <v>1.75</v>
       </c>
       <c r="K66" s="14">
         <f t="shared" si="3"/>
-        <v>0.63111111111111107</v>
+        <v>0.35</v>
       </c>
       <c r="M66">
         <f t="shared" si="4"/>
-        <v>28.4</v>
+        <v>17.5</v>
       </c>
       <c r="N66">
         <f t="shared" si="10"/>
-        <v>5.68</v>
+        <v>3.4999999999999996</v>
       </c>
       <c r="O66">
         <f t="shared" si="11"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P66">
         <f t="shared" si="12"/>
@@ -6899,7 +6899,7 @@
       </c>
       <c r="R66">
         <f t="shared" si="16"/>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="67" spans="1:18" x14ac:dyDescent="0.25">
@@ -7221,7 +7221,7 @@
     <col min="8" max="28" width="6.28515625" style="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>140</v>
       </c>
@@ -7229,7 +7229,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="13"/>
       <c r="B2" t="s">
         <v>136</v>
@@ -7253,21 +7253,21 @@
         <v>141</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>132</v>
       </c>
       <c r="B3">
         <f>SUM(H3:AB3)</f>
-        <v>0</v>
+        <v>-22</v>
       </c>
       <c r="C3">
         <f>(B3/$C$1)*100</f>
-        <v>0</v>
+        <v>-4.3999999999999995</v>
       </c>
       <c r="D3">
         <f>COUNTA(H3:AB3)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <f>COUNTIF(H3:AB3, "&gt;0")</f>
@@ -7279,10 +7279,13 @@
       </c>
       <c r="G3">
         <f>COUNTIF(H3:AB3, "&lt;0")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="H3" s="15">
+        <v>-22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>100</v>
       </c>
@@ -7311,21 +7314,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>135</v>
       </c>
       <c r="B5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-18.2</v>
       </c>
       <c r="C5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-3.64</v>
       </c>
       <c r="D5">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E5">
         <f t="shared" si="3"/>
@@ -7337,10 +7340,16 @@
       </c>
       <c r="G5">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="H5" s="15">
+        <v>-4.2</v>
+      </c>
+      <c r="I5" s="15">
+        <v>-14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>133</v>
       </c>
@@ -7369,25 +7378,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>134</v>
       </c>
       <c r="B7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="C7">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="D7">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7">
         <f t="shared" si="4"/>
@@ -7397,8 +7406,11 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H7" s="15">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>74</v>
       </c>
@@ -7427,7 +7439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>99</v>
       </c>
@@ -7456,7 +7468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>101</v>
       </c>
@@ -7485,7 +7497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>77</v>
       </c>
@@ -7514,25 +7526,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>72</v>
       </c>
       <c r="B12">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-10.900000000000002</v>
       </c>
       <c r="C12">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-2.1800000000000002</v>
       </c>
       <c r="D12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E12">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12">
         <f t="shared" si="4"/>
@@ -7540,10 +7552,19 @@
       </c>
       <c r="G12">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="H12" s="15">
+        <v>0.6</v>
+      </c>
+      <c r="I12" s="15">
+        <v>-9.3000000000000007</v>
+      </c>
+      <c r="J12" s="15">
+        <v>-2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>102</v>
       </c>
@@ -7572,7 +7593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>76</v>
       </c>
@@ -7601,25 +7622,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>60</v>
       </c>
       <c r="B15">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-12.4</v>
       </c>
       <c r="C15">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-2.48</v>
       </c>
       <c r="D15">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E15">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15">
         <f t="shared" si="4"/>
@@ -7627,28 +7648,34 @@
       </c>
       <c r="G15">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="H15" s="15">
+        <v>-17.5</v>
+      </c>
+      <c r="I15" s="15">
+        <v>5.0999999999999996</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>67</v>
       </c>
       <c r="B16">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="C16">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.88</v>
       </c>
       <c r="D16">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16">
         <f t="shared" si="4"/>
@@ -7658,8 +7685,11 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H16" s="15">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>94</v>
       </c>
@@ -7688,7 +7718,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>95</v>
       </c>
@@ -7717,7 +7747,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>65</v>
       </c>
@@ -7746,7 +7776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>103</v>
       </c>
@@ -7775,25 +7805,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>69</v>
       </c>
       <c r="B21">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C21">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="D21">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E21">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F21">
         <f t="shared" si="4"/>
@@ -7803,8 +7833,14 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H21" s="15">
+        <v>1.3</v>
+      </c>
+      <c r="I21" s="15">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>85</v>
       </c>
@@ -7833,21 +7869,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>121</v>
       </c>
       <c r="B23">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-3.1</v>
       </c>
       <c r="C23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-0.62</v>
       </c>
       <c r="D23">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23">
         <f t="shared" si="3"/>
@@ -7859,24 +7895,27 @@
       </c>
       <c r="G23">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="H23" s="15">
+        <v>-3.1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>66</v>
       </c>
       <c r="B24">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-2.4</v>
       </c>
       <c r="C24">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-0.48</v>
       </c>
       <c r="D24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24">
         <f t="shared" si="3"/>
@@ -7888,10 +7927,13 @@
       </c>
       <c r="G24">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="H24" s="15">
+        <v>-2.4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>120</v>
       </c>
@@ -7920,7 +7962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>122</v>
       </c>
@@ -7949,7 +7991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>123</v>
       </c>
@@ -7978,25 +8020,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>70</v>
       </c>
       <c r="B28">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-5.5</v>
       </c>
       <c r="C28">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-1.0999999999999999</v>
       </c>
       <c r="D28">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E28">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F28">
         <f t="shared" si="4"/>
@@ -8004,10 +8046,25 @@
       </c>
       <c r="G28">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+      <c r="H28" s="15">
+        <v>3.7</v>
+      </c>
+      <c r="I28" s="15">
+        <v>-1.2</v>
+      </c>
+      <c r="J28" s="15">
+        <v>-0.9</v>
+      </c>
+      <c r="K28" s="15">
+        <v>-4</v>
+      </c>
+      <c r="L28" s="15">
+        <v>-3.1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>130</v>
       </c>
@@ -8036,7 +8093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>64</v>
       </c>
@@ -8065,21 +8122,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>128</v>
       </c>
       <c r="B31">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-3.8</v>
       </c>
       <c r="C31">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-0.76</v>
       </c>
       <c r="D31">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E31">
         <f t="shared" si="3"/>
@@ -8091,10 +8148,13 @@
       </c>
       <c r="G31">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="H31" s="15">
+        <v>-3.8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>126</v>
       </c>
@@ -8123,25 +8183,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>124</v>
       </c>
       <c r="B33">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="C33">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="D33">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E33">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F33">
         <f t="shared" si="4"/>
@@ -8151,26 +8211,29 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H33" s="15">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>127</v>
       </c>
       <c r="B34">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="C34">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.76</v>
       </c>
       <c r="D34">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E34">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F34">
         <f t="shared" si="4"/>
@@ -8180,8 +8243,11 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H34" s="15">
+        <v>8.8000000000000007</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>129</v>
       </c>
@@ -8210,21 +8276,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>131</v>
       </c>
       <c r="B36">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-2.7</v>
       </c>
       <c r="C36">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-0.54</v>
       </c>
       <c r="D36">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E36">
         <f t="shared" si="3"/>
@@ -8236,10 +8302,13 @@
       </c>
       <c r="G36">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="H36" s="15">
+        <v>-2.7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>117</v>
       </c>
@@ -8268,7 +8337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>98</v>
       </c>
@@ -8297,7 +8366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>86</v>
       </c>
@@ -8326,7 +8395,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>68</v>
       </c>
@@ -8355,21 +8424,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>87</v>
       </c>
       <c r="B41">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-3.1</v>
       </c>
       <c r="C41">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-0.62</v>
       </c>
       <c r="D41">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E41">
         <f t="shared" si="3"/>
@@ -8381,10 +8450,13 @@
       </c>
       <c r="G41">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="H41" s="15">
+        <v>-3.1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>118</v>
       </c>
@@ -8413,7 +8485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>119</v>
       </c>
@@ -8442,7 +8514,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>125</v>
       </c>
@@ -8471,21 +8543,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>79</v>
       </c>
       <c r="B45">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-10.5</v>
       </c>
       <c r="C45">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-2.1</v>
       </c>
       <c r="D45">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E45">
         <f t="shared" si="3"/>
@@ -8497,10 +8569,13 @@
       </c>
       <c r="G45">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="H45" s="15">
+        <v>-10.5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>106</v>
       </c>
@@ -8529,7 +8604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>97</v>
       </c>
@@ -8558,7 +8633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>105</v>
       </c>
@@ -8587,7 +8662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>54</v>
       </c>
@@ -8616,7 +8691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>75</v>
       </c>
@@ -8645,21 +8720,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>108</v>
       </c>
       <c r="B51">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="C51">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="D51">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E51">
         <f t="shared" si="3"/>
@@ -8671,10 +8746,13 @@
       </c>
       <c r="G51">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="H51" s="15">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>71</v>
       </c>
@@ -8703,7 +8781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>107</v>
       </c>
@@ -8732,21 +8810,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>78</v>
       </c>
       <c r="B54">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-4.5999999999999996</v>
       </c>
       <c r="C54">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-0.91999999999999993</v>
       </c>
       <c r="D54">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E54">
         <f t="shared" si="3"/>
@@ -8758,10 +8836,13 @@
       </c>
       <c r="G54">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="H54" s="15">
+        <v>-4.5999999999999996</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>109</v>
       </c>
@@ -8790,25 +8871,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>73</v>
       </c>
       <c r="B56">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>7.4</v>
       </c>
       <c r="C56">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.48</v>
       </c>
       <c r="D56">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E56">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F56">
         <f t="shared" si="4"/>
@@ -8818,8 +8899,11 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H56" s="15">
+        <v>7.4</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>114</v>
       </c>
@@ -8848,7 +8932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>110</v>
       </c>
@@ -8877,7 +8961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>111</v>
       </c>
@@ -8906,7 +8990,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>113</v>
       </c>
@@ -8935,7 +9019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>115</v>
       </c>
@@ -8964,7 +9048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>112</v>
       </c>
@@ -8993,7 +9077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>116</v>
       </c>
@@ -9022,21 +9106,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>62</v>
       </c>
       <c r="B64">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-17.100000000000001</v>
       </c>
       <c r="C64">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-3.42</v>
       </c>
       <c r="D64">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E64">
         <f t="shared" si="3"/>
@@ -9048,28 +9132,31 @@
       </c>
       <c r="G64">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="H64" s="15">
+        <v>-17.100000000000001</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>61</v>
       </c>
       <c r="B65">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-2.9</v>
       </c>
       <c r="C65">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-0.57999999999999996</v>
       </c>
       <c r="D65">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E65">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F65">
         <f t="shared" si="4"/>
@@ -9077,10 +9164,19 @@
       </c>
       <c r="G65">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="H65" s="15">
+        <v>-7</v>
+      </c>
+      <c r="I65" s="15">
+        <v>4.2</v>
+      </c>
+      <c r="J65" s="15">
+        <v>-0.1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>96</v>
       </c>
@@ -9109,21 +9205,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>63</v>
       </c>
       <c r="B67">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-10.9</v>
       </c>
       <c r="C67">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-2.1800000000000002</v>
       </c>
       <c r="D67">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E67">
         <f t="shared" si="3"/>
@@ -9135,10 +9231,13 @@
       </c>
       <c r="G67">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="H67" s="15">
+        <v>-10.9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>104</v>
       </c>

</xml_diff>